<commit_message>
auto: remove sold items
</commit_message>
<xml_diff>
--- a/CS_GO_PnL_Tracker_Final.xlsx
+++ b/CS_GO_PnL_Tracker_Final.xlsx
@@ -230,7 +230,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -375,6 +375,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -8525,26 +8546,32 @@
       <c r="H230" s="53" t="n"/>
     </row>
     <row r="231" ht="19.5" customHeight="1">
-      <c r="A231" s="10" t="n"/>
-      <c r="B231" s="27" t="n"/>
-      <c r="C231" s="34" t="n"/>
-      <c r="D231" s="11">
-        <f>IF(C231="","",C231*$B$1)</f>
-        <v/>
-      </c>
-      <c r="E231" s="12">
-        <f>IF(C231="","",C231-D231)</f>
-        <v/>
-      </c>
-      <c r="F231" s="19">
-        <f>IF(OR(B231="",C231=""),"",E231-B231)</f>
-        <v/>
-      </c>
-      <c r="G231" s="22">
-        <f>IF(OR(B231="",B231=0),"",F231/B231)</f>
-        <v/>
-      </c>
-      <c r="H231" s="13" t="n"/>
+      <c r="A231" s="45" t="inlineStr">
+        <is>
+          <t>MAG-7 | Sand Dune .152819916606</t>
+        </is>
+      </c>
+      <c r="B231" s="54" t="n"/>
+      <c r="C231" s="55" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D231" s="56">
+        <f>C231*$B$1</f>
+        <v/>
+      </c>
+      <c r="E231" s="57">
+        <f>C231-D231</f>
+        <v/>
+      </c>
+      <c r="F231" s="58">
+        <f>E231-B231</f>
+        <v/>
+      </c>
+      <c r="G231" s="59">
+        <f>F231/B231</f>
+        <v/>
+      </c>
+      <c r="H231" s="60" t="n"/>
     </row>
     <row r="232" ht="19.5" customHeight="1">
       <c r="A232" s="6" t="n"/>

</xml_diff>